<commit_message>
feat: rebuild Nanosurf and Ametek Brookfield product pages verbatim from Drive docs, with opt-in fields for typed tool inputs, verbatim symbols and multi-column specs
</commit_message>
<xml_diff>
--- a/outputs/Inkarp_Solution_Finder_Improvement_Plan.xlsx
+++ b/outputs/Inkarp_Solution_Finder_Improvement_Plan.xlsx
@@ -1,22 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sharath\Desktop\Inkarp-Nextjs\outputs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="12" windowWidth="16092" windowHeight="9660" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Detailed Plan" sheetId="2" r:id="rId2"/>
     <sheet name="Roadmap" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="287">
   <si>
     <t>Inkarp Homepage Solution Finder — Improvement Plan</t>
   </si>
@@ -882,8 +887,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1018,8 +1023,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1028,10 +1049,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1042,20 +1059,22 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1067,19 +1086,16 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1149,7 +1165,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1181,9 +1197,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1215,6 +1232,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1390,258 +1408,258 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="8" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="4.6640625" customWidth="1"/>
+    <col min="4" max="8" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="4" t="s">
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <f>COUNTA('Detailed Plan'!A5:A26)</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="4" t="s">
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+    </row>
+    <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="3">
         <f>COUNTIF('Detailed Plan'!H5:H26,"High")</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+    </row>
+    <row r="7" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="3">
         <f>COUNTIF('Detailed Plan'!H5:H26,"Medium")</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+    </row>
+    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <f>COUNTIF('Detailed Plan'!J5:J26,"Now (0–2 weeks)")</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="4" t="s">
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="3">
         <f>COUNTIF('Detailed Plan'!J5:J26,"Next (2–6 weeks)")</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5">
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
         <f>COUNTIF('Detailed Plan'!J5:J26,"Later (6–12 weeks)")</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="8" t="s">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A13:H15"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="D4:H4"/>
     <mergeCell ref="D5:H7"/>
     <mergeCell ref="D8:H10"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A13:H15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="4" width="29.7109375" customWidth="1"/>
-    <col min="5" max="5" width="26.7109375" customWidth="1"/>
-    <col min="6" max="6" width="34.7109375" customWidth="1"/>
-    <col min="7" max="7" width="33.7109375" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19.7109375" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" customWidth="1"/>
-    <col min="12" max="12" width="27.7109375" customWidth="1"/>
-    <col min="13" max="13" width="28.7109375" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" customWidth="1"/>
+    <col min="3" max="4" width="29.6640625" customWidth="1"/>
+    <col min="5" max="5" width="26.6640625" customWidth="1"/>
+    <col min="6" max="6" width="34.6640625" customWidth="1"/>
+    <col min="7" max="7" width="33.6640625" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" customWidth="1"/>
+    <col min="10" max="10" width="19.6640625" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" customWidth="1"/>
+    <col min="12" max="12" width="27.6640625" customWidth="1"/>
+    <col min="13" max="13" width="28.6640625" customWidth="1"/>
+    <col min="14" max="14" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="30" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-    </row>
-    <row r="2" spans="1:14" ht="28" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+    </row>
+    <row r="2" spans="1:14" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-    </row>
-    <row r="4" spans="1:14">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1685,971 +1703,971 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="76" customHeight="1">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="M5" s="10" t="s">
+      <c r="M5" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="N5" s="11" t="s">
+      <c r="N5" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="76" customHeight="1">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="K6" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="M6" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="76" customHeight="1">
-      <c r="A7" s="9" t="s">
+    <row r="7" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="M7" s="10" t="s">
+      <c r="M7" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="N7" s="11" t="s">
+      <c r="N7" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="76" customHeight="1">
-      <c r="A8" s="9" t="s">
+    <row r="8" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="K8" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="M8" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="76" customHeight="1">
-      <c r="A9" s="9" t="s">
+    <row r="9" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="K9" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="M9" s="10" t="s">
+      <c r="M9" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="N9" s="11" t="s">
+      <c r="N9" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="76" customHeight="1">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K10" s="10" t="s">
+      <c r="K10" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="L10" s="10" t="s">
+      <c r="L10" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="M10" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="76" customHeight="1">
-      <c r="A11" s="9" t="s">
+    <row r="11" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="10" t="s">
+      <c r="K11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="L11" s="10" t="s">
+      <c r="L11" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="M11" s="10" t="s">
+      <c r="M11" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="11" t="s">
+      <c r="N11" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="76" customHeight="1">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="K12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="L12" s="10" t="s">
+      <c r="L12" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="M12" s="10" t="s">
+      <c r="M12" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="N12" s="11" t="s">
+      <c r="N12" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="76" customHeight="1">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K13" s="10" t="s">
+      <c r="K13" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="L13" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="M13" s="10" t="s">
+      <c r="M13" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="N13" s="11" t="s">
+      <c r="N13" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="76" customHeight="1">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J14" s="10" t="s">
+      <c r="J14" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="L14" s="10" t="s">
+      <c r="L14" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="M14" s="10" t="s">
+      <c r="M14" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="N14" s="11" t="s">
+      <c r="N14" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="76" customHeight="1">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="G15" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J15" s="10" t="s">
+      <c r="J15" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K15" s="10" t="s">
+      <c r="K15" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="L15" s="10" t="s">
+      <c r="L15" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="M15" s="10" t="s">
+      <c r="M15" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="N15" s="11" t="s">
+      <c r="N15" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="76" customHeight="1">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I16" s="10" t="s">
+      <c r="I16" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="J16" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K16" s="10" t="s">
+      <c r="K16" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="L16" s="10" t="s">
+      <c r="L16" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="M16" s="10" t="s">
+      <c r="M16" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="N16" s="11" t="s">
+      <c r="N16" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="76" customHeight="1">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="I17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J17" s="10" t="s">
+      <c r="J17" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K17" s="10" t="s">
+      <c r="K17" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="L17" s="10" t="s">
+      <c r="L17" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="M17" s="10" t="s">
+      <c r="M17" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="N17" s="11" t="s">
+      <c r="N17" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="76" customHeight="1">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K18" s="10" t="s">
+      <c r="K18" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="L18" s="10" t="s">
+      <c r="L18" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="M18" s="10" t="s">
+      <c r="M18" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="N18" s="11" t="s">
+      <c r="N18" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="76" customHeight="1">
-      <c r="A19" s="9" t="s">
+    <row r="19" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="J19" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K19" s="10" t="s">
+      <c r="K19" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="L19" s="10" t="s">
+      <c r="L19" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="M19" s="10" t="s">
+      <c r="M19" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="N19" s="11" t="s">
+      <c r="N19" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="76" customHeight="1">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J20" s="10" t="s">
+      <c r="J20" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K20" s="10" t="s">
+      <c r="K20" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="L20" s="10" t="s">
+      <c r="L20" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="M20" s="10" t="s">
+      <c r="M20" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="N20" s="11" t="s">
+      <c r="N20" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="76" customHeight="1">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="I21" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J21" s="10" t="s">
+      <c r="J21" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K21" s="10" t="s">
+      <c r="K21" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="L21" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="M21" s="10" t="s">
+      <c r="M21" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="N21" s="11" t="s">
+      <c r="N21" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="76" customHeight="1">
-      <c r="A22" s="9" t="s">
+    <row r="22" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="H22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="I22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J22" s="10" t="s">
+      <c r="J22" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="L22" s="10" t="s">
+      <c r="L22" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="M22" s="10" t="s">
+      <c r="M22" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="N22" s="11" t="s">
+      <c r="N22" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="76" customHeight="1">
-      <c r="A23" s="9" t="s">
+    <row r="23" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G23" s="10" t="s">
+      <c r="G23" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I23" s="10" t="s">
+      <c r="I23" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J23" s="10" t="s">
+      <c r="J23" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K23" s="10" t="s">
+      <c r="K23" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="L23" s="10" t="s">
+      <c r="L23" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="M23" s="10" t="s">
+      <c r="M23" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="N23" s="11" t="s">
+      <c r="N23" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="76" customHeight="1">
-      <c r="A24" s="9" t="s">
+    <row r="24" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="I24" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J24" s="10" t="s">
+      <c r="J24" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K24" s="10" t="s">
+      <c r="K24" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="L24" s="10" t="s">
+      <c r="L24" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="M24" s="10" t="s">
+      <c r="M24" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="N24" s="11" t="s">
+      <c r="N24" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="76" customHeight="1">
-      <c r="A25" s="9" t="s">
+    <row r="25" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="G25" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J25" s="10" t="s">
+      <c r="J25" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K25" s="10" t="s">
+      <c r="K25" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="L25" s="10" t="s">
+      <c r="L25" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="M25" s="10" t="s">
+      <c r="M25" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="N25" s="11" t="s">
+      <c r="N25" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="76" customHeight="1">
-      <c r="A26" s="9" t="s">
+    <row r="26" spans="1:14" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J26" s="10" t="s">
+      <c r="J26" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="K26" s="10" t="s">
+      <c r="K26" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="L26" s="10" t="s">
+      <c r="L26" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="M26" s="10" t="s">
+      <c r="M26" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="N26" s="11" t="s">
+      <c r="N26" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2659,12 +2677,12 @@
     <mergeCell ref="A2:N2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H26">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",H5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J26">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>LEFT(J5,3)="Now"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2681,210 +2699,210 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="30.7109375" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" customWidth="1"/>
-    <col min="7" max="7" width="34.7109375" customWidth="1"/>
-    <col min="8" max="8" width="29.7109375" customWidth="1"/>
+    <col min="1" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30.6640625" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" customWidth="1"/>
+    <col min="7" max="7" width="34.6640625" customWidth="1"/>
+    <col min="8" max="8" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="92" customHeight="1">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:8" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="5" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="92" customHeight="1">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:8" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="5" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="92" customHeight="1">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:8" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="5" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <f>COUNTIF('Detailed Plan'!J5:J26,A10)</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="5">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3">
         <f>COUNTIFS('Detailed Plan'!J5:J26,A10,'Detailed Plan'!H5:H26,"High")</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="5">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3">
         <f>COUNTIFS('Detailed Plan'!J5:J26,A10,'Detailed Plan'!H5:H26,"Medium")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="3">
         <f>COUNTIF('Detailed Plan'!J5:J26,A11)</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="5">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3">
         <f>COUNTIFS('Detailed Plan'!J5:J26,A11,'Detailed Plan'!H5:H26,"High")</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="5">
+        <v>5</v>
+      </c>
+      <c r="D11" s="3">
         <f>COUNTIFS('Detailed Plan'!J5:J26,A11,'Detailed Plan'!H5:H26,"Medium")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="3">
         <f>COUNTIF('Detailed Plan'!J5:J26,A12)</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="5">
+        <v>3</v>
+      </c>
+      <c r="C12" s="3">
         <f>COUNTIFS('Detailed Plan'!J5:J26,A12,'Detailed Plan'!H5:H26,"High")</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3">
         <f>COUNTIFS('Detailed Plan'!J5:J26,A12,'Detailed Plan'!H5:H26,"Medium")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>